<commit_message>
Seed TCs_improved for the boards case
The same treatment the wiring case had: an exact copy of TCs, 52 rows, and
improvement_start 2030 / improvement_end 2060 in the source sheet. Every seeded
row says in its source column that it is a copy and NOT an improvement, to be
replaced with the number that process reaches once improved.

Checked, not assumed: the deterministic solution is 1,650 rows before and after,
every row matching, worst absolute difference exactly 0. The ramp is live all
the same -- 572 rows, 11 years x 52 coefficients, Year column present, no
duplicated (year, coefficient) pair.

carcomposition_mockup is deliberately NOT seeded. Its coefficients are generated
by make_carcomposition_tcs.py and every one is MADE UP; seeding it would be
filling invented numbers with invented numbers, and there is nobody waiting to
type real ones into it.

All 10 checks pass.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data_folder/bev_electronics_boards/input_data/case.xlsx
+++ b/data_folder/bev_electronics_boards/input_data/case.xlsx
@@ -11,6 +11,7 @@
     <sheet name="_lists" sheetId="2" state="hidden" r:id="rId2"/>
     <sheet name="processes" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="TCs" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="TCs_improved" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -426,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -523,6 +524,7 @@
           <t>material_suffix</t>
         </is>
       </c>
+      <c r="B8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -545,6 +547,30 @@
       <c r="B10" t="inlineStr">
         <is>
           <t>200000</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>improvement_start</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2030</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>improvement_end</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2060</t>
         </is>
       </c>
     </row>
@@ -4306,4 +4332,3258 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L53"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Input_FlowID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Input_layer</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Input_layer_key</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Output_FlowID</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>TC_target_layer</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>TC_target_key</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>value_min</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>value_max</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>technology</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>F_collected</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>product</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>BEV</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PCB</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0.6</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0.45</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>disassembly</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- a main board is a discrete part in a known place, so a worker looking for it finds it.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>F_collected</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>product</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>BEV</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>F_in_car</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PCB</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>0.28</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>0.52</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>disassembly</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- NOT AN INDEPENDENT MEASUREMENT: it is 1 minus what left in the stream, given its own range. Replace it with a number measured on this side.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>F_in_car</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>product</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>BEV</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>F_shredded</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PCB</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>stays_in_car</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>definitional</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: DEFINITIONAL: the car goes to the shredder, so what is in it goes too.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>F_collected</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>product</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>BEV</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>0.15</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>disassembly</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- sensors are scattered through the car in tens of places and most are never sought.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>F_collected</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>product</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>BEV</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>F_in_car</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>0.49</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>0.76</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>disassembly</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- NOT AN INDEPENDENT MEASUREMENT: it is 1 minus what left in the stream, given its own range. Replace it with a number measured on this side.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>F_in_car</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>product</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>BEV</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>F_shredded</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>stays_in_car</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>definitional</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: DEFINITIONAL: the car goes to the shredder, so what is in it goes too.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>PCB</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>F_recovered_own</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Ag</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- what the specialist route is built around: its own process, and a price that pays for it.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>PCB</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>F_loss_own</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Ag</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>0.035</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>0.24</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- NOT AN INDEPENDENT MEASUREMENT: it is 1 minus what left in the stream, given its own range. Replace it with a number measured on this side.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>PCB</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>F_recovered_own</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Au</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- what the specialist route is built around: its own process, and a price that pays for it.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>PCB</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>F_loss_own</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Au</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>0.035</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>0.24</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- NOT AN INDEPENDENT MEASUREMENT: it is 1 minus what left in the stream, given its own range. Replace it with a number measured on this side.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>PCB</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>F_recovered_own</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Cu</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- what the specialist route is built around: its own process, and a price that pays for it.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>PCB</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>F_loss_own</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Cu</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>0.07</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>0.28</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- NOT AN INDEPENDENT MEASUREMENT: it is 1 minus what left in the stream, given its own range. Replace it with a number measured on this side.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>PCB</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>F_recovered_own</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Ni</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>0.85</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>0.65</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- collected with the copper rather than by a process of its own.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>PCB</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>F_loss_own</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Ni</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>0.15</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>0.105</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>0.32</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- NOT AN INDEPENDENT MEASUREMENT: it is 1 minus what left in the stream, given its own range. Replace it with a number measured on this side.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>PCB</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>F_recovered_own</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Pd</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- what the specialist route is built around: its own process, and a price that pays for it.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>PCB</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>F_loss_own</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Pd</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>0.035</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>0.24</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- NOT AN INDEPENDENT MEASUREMENT: it is 1 minus what left in the stream, given its own range. Replace it with a number measured on this side.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>F_recovered_own</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Ag</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- what the specialist route is built around: its own process, and a price that pays for it.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>F_loss_own</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Ag</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>0.035</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>0.24</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- NOT AN INDEPENDENT MEASUREMENT: it is 1 minus what left in the stream, given its own range. Replace it with a number measured on this side.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>F_recovered_own</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Au</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- what the specialist route is built around: its own process, and a price that pays for it.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>F_loss_own</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Au</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>0.035</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>0.24</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- NOT AN INDEPENDENT MEASUREMENT: it is 1 minus what left in the stream, given its own range. Replace it with a number measured on this side.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>F_recovered_own</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: Boron is not recovered: no process at this scale separates a trace dopant out of a ground board. Written as a definite 0 with NO range, like `rest`, rather than 0 with a band up to 0.1 -- that band said "maybe a tenth of it" on no evidence at all, and it left this group with one ranged row against one fixed one, which src/sampling.py rightly refuses: the constraint pins the loss at 1 - B, so B's range would be discarded without a word.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>F_loss_own</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- NOT AN INDEPENDENT MEASUREMENT: it is 1 minus what left in the stream, given its own range. Replace it with a number measured on this side.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>F_recovered_own</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Co</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>0.6</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- collected with the copper rather than by a process of its own.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>F_loss_own</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Co</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>0.28</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>0.52</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- NOT AN INDEPENDENT MEASUREMENT: it is 1 minus what left in the stream, given its own range. Replace it with a number measured on this side.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>F_recovered_own</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Cu</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- what the specialist route is built around: its own process, and a price that pays for it.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>F_loss_own</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Cu</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>0.07</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>0.28</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- NOT AN INDEPENDENT MEASUREMENT: it is 1 minus what left in the stream, given its own range. Replace it with a number measured on this side.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>F_recovered_own</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Dy</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>0.15</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- no process of its own at this scale; it goes to the slag.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>F_loss_own</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Dy</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>0.665</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- NOT AN INDEPENDENT MEASUREMENT: it is 1 minus what left in the stream, given its own range. Replace it with a number measured on this side.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>F_recovered_own</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Ga</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>0.02</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>0.12</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- no process of its own at this scale; it goes to the slag.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>F_loss_own</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Ga</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>0.98</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>0.686</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>0.984</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- NOT AN INDEPENDENT MEASUREMENT: it is 1 minus what left in the stream, given its own range. Replace it with a number measured on this side.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>F_recovered_own</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Ge</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>0.02</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>0.12</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- no process of its own at this scale; it goes to the slag.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>F_loss_own</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Ge</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>0.98</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>0.686</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>0.984</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- NOT AN INDEPENDENT MEASUREMENT: it is 1 minus what left in the stream, given its own range. Replace it with a number measured on this side.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>F_recovered_own</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>In</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>0.15</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- no process of its own at this scale; it goes to the slag.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>F_loss_own</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>In</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>0.665</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- NOT AN INDEPENDENT MEASUREMENT: it is 1 minus what left in the stream, given its own range. Replace it with a number measured on this side.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>F_recovered_own</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Li</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>0.15</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- no process of its own at this scale; it goes to the slag.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>F_loss_own</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Li</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>0.665</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- NOT AN INDEPENDENT MEASUREMENT: it is 1 minus what left in the stream, given its own range. Replace it with a number measured on this side.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>F_recovered_own</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Mn</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>0.15</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- no process of its own at this scale; it goes to the slag.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>F_loss_own</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Mn</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>0.665</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- NOT AN INDEPENDENT MEASUREMENT: it is 1 minus what left in the stream, given its own range. Replace it with a number measured on this side.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>F_recovered_own</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Nd</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>0.15</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- no process of its own at this scale; it goes to the slag.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>F_loss_own</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Nd</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>0.665</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- NOT AN INDEPENDENT MEASUREMENT: it is 1 minus what left in the stream, given its own range. Replace it with a number measured on this side.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>F_recovered_own</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Ni</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>0.85</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>0.65</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- collected with the copper rather than by a process of its own.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>F_loss_own</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Ni</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>0.15</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>0.105</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>0.32</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- NOT AN INDEPENDENT MEASUREMENT: it is 1 minus what left in the stream, given its own range. Replace it with a number measured on this side.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>F_recovered_own</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Pt</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- what the specialist route is built around: its own process, and a price that pays for it.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>F_loss_own</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Pt</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>0.035</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>0.24</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- NOT AN INDEPENDENT MEASUREMENT: it is 1 minus what left in the stream, given its own range. Replace it with a number measured on this side.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>F_recovered_own</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Ta</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- no process of its own at this scale; it goes to the slag.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>F_loss_own</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Ta</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>0.63</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>0.92</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- NOT AN INDEPENDENT MEASUREMENT: it is 1 minus what left in the stream, given its own range. Replace it with a number measured on this side.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>F_recovered_own</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Ti</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>0.02</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>0.12</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- no process of its own at this scale; it goes to the slag.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>F_loss_own</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Ti</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>0.98</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>0.686</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>0.984</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- NOT AN INDEPENDENT MEASUREMENT: it is 1 minus what left in the stream, given its own range. Replace it with a number measured on this side.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>F_recovered_own</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>0.15</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- no process of its own at this scale; it goes to the slag.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>F_loss_own</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>0.665</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: PLACEHOLDER (Claude, not data) -- NOT AN INDEPENDENT MEASUREMENT: it is 1 minus what left in the stream, given its own range. Replace it with a number measured on this side.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>PCB</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>F_loss_own</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>rest</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: Unspecified material -- board laminate, plastics. Not recovered.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>F_disassembled</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Sensors</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>F_loss_own</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>material</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>rest</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>specialist_recycling</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>grinding_then_element</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>SEEDED COPY of the current value -- NOT an improvement. Replace with the number this process reaches once improved, and its range. Until you do, this case ramps from a value to itself and every year is identical. (was: Unspecified material -- board laminate, plastics. Not recovered.)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>